<commit_message>
Actualizacion automatica de datos - vie 05/06/2026 16:11:59,20
</commit_message>
<xml_diff>
--- a/Teletrabajo/Teletrabajo.xlsx
+++ b/Teletrabajo/Teletrabajo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Teletrabajo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFDE3343-B6A1-4EAA-B152-95F8A5A24219}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5679F156-F030-402E-B53D-FD49DA3732CF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
   </bookViews>
   <sheets>
     <sheet name="Teletrabajo" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="36">
   <si>
     <t>Josue</t>
   </si>
@@ -284,17 +284,17 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -630,52 +630,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B5EDDC-5ADB-4A4C-9736-3AC62D35C32F}">
-  <dimension ref="A1:Q36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="18.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Q33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="18.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.88671875" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.5546875" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="3.88671875" customWidth="1"/>
-    <col min="14" max="14" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.6640625" customWidth="1"/>
-    <col min="17" max="17" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.6640625" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.5703125" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="3.85546875" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.7109375" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="D1" s="7" t="s">
+      <c r="B1" s="10"/>
+      <c r="D1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="8"/>
-      <c r="G1" s="7" t="s">
+      <c r="E1" s="10"/>
+      <c r="G1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="8"/>
-      <c r="J1" s="7" t="s">
+      <c r="H1" s="10"/>
+      <c r="J1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="8"/>
-      <c r="M1" s="7" t="s">
+      <c r="K1" s="10"/>
+      <c r="M1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="8"/>
-      <c r="P1" s="7" t="s">
+      <c r="N1" s="10"/>
+      <c r="P1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Q1" s="8"/>
-    </row>
-    <row r="2" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q1" s="10"/>
+    </row>
+    <row r="2" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>24</v>
       </c>
@@ -713,7 +713,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -751,7 +751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -789,7 +789,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -827,7 +827,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -865,7 +865,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -903,7 +903,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -941,7 +941,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
@@ -973,7 +973,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G10" s="1" t="s">
         <v>13</v>
       </c>
@@ -999,7 +999,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="J11" s="1" t="s">
         <v>13</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="J12" s="1" t="s">
         <v>14</v>
       </c>
@@ -1039,29 +1039,29 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="D14" s="7" t="s">
+      <c r="B14" s="10"/>
+      <c r="D14" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="8"/>
-      <c r="G14" s="7" t="s">
+      <c r="E14" s="10"/>
+      <c r="G14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="J14" s="7" t="s">
+      <c r="H14" s="10"/>
+      <c r="J14" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="K14" s="8"/>
-      <c r="M14" s="7" t="s">
+      <c r="K14" s="10"/>
+      <c r="M14" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="N14" s="8"/>
-    </row>
-    <row r="15" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="N14" s="10"/>
+    </row>
+    <row r="15" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>24</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
@@ -1221,7 +1221,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>0</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>2</v>
       </c>
@@ -1347,73 +1347,49 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="9" t="s">
+    <row r="28" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="9"/>
-    </row>
-    <row r="29" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="10" t="s">
+      <c r="B28" s="8"/>
+    </row>
+    <row r="29" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="10" t="s">
-        <v>15</v>
+    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>2</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="B36" s="2" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 17/07/2026 18:05:52,90
</commit_message>
<xml_diff>
--- a/Teletrabajo/Teletrabajo.xlsx
+++ b/Teletrabajo/Teletrabajo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Teletrabajo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5679F156-F030-402E-B53D-FD49DA3732CF}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD344004-E672-4E4D-973E-F89CC4129A16}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
   </bookViews>
   <sheets>
     <sheet name="Teletrabajo" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="37">
   <si>
     <t>Josue</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>Miecoles</t>
+  </si>
+  <si>
+    <t>Semana del 21 - 24 de Julio</t>
   </si>
 </sst>
 </file>
@@ -631,25 +634,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B5EDDC-5ADB-4A4C-9736-3AC62D35C32F}">
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="18.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="18.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.85546875" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.5703125" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="3.85546875" customWidth="1"/>
-    <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.7109375" customWidth="1"/>
-    <col min="17" max="17" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.88671875" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.5546875" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="3.88671875" customWidth="1"/>
+    <col min="14" max="14" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.6640625" customWidth="1"/>
+    <col min="17" max="17" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>18</v>
       </c>
@@ -675,7 +678,7 @@
       </c>
       <c r="Q1" s="10"/>
     </row>
-    <row r="2" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>24</v>
       </c>
@@ -713,7 +716,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -751,7 +754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -789,7 +792,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -827,7 +830,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -865,7 +868,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -903,7 +906,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -941,7 +944,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
@@ -973,7 +976,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="G10" s="1" t="s">
         <v>13</v>
       </c>
@@ -999,7 +1002,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="J11" s="1" t="s">
         <v>13</v>
       </c>
@@ -1019,7 +1022,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="J12" s="1" t="s">
         <v>14</v>
       </c>
@@ -1039,7 +1042,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>17</v>
       </c>
@@ -1061,7 +1064,7 @@
       </c>
       <c r="N14" s="10"/>
     </row>
-    <row r="15" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>24</v>
       </c>
@@ -1093,7 +1096,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1125,7 +1128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1157,7 +1160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -1189,7 +1192,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
@@ -1221,7 +1224,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
@@ -1253,7 +1256,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
@@ -1285,7 +1288,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -1311,7 +1314,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>0</v>
       </c>
@@ -1331,7 +1334,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -1339,7 +1342,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>2</v>
       </c>
@@ -1347,37 +1350,59 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B28" s="8"/>
-    </row>
-    <row r="29" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D28" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28" s="8"/>
+    </row>
+    <row r="29" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D29" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>16</v>
       </c>
@@ -1385,7 +1410,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>2</v>
       </c>
@@ -1394,7 +1419,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="P1:Q1"/>
@@ -1407,6 +1432,7 @@
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="M14:N14"/>
+    <mergeCell ref="D28:E28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - mar 21/07/2026  8:53:28,26
</commit_message>
<xml_diff>
--- a/Teletrabajo/Teletrabajo.xlsx
+++ b/Teletrabajo/Teletrabajo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Teletrabajo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD344004-E672-4E4D-973E-F89CC4129A16}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A18DD47B-BA3C-4AF2-9299-2EA07C47029C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
   </bookViews>
   <sheets>
     <sheet name="Teletrabajo" sheetId="1" r:id="rId1"/>
@@ -634,25 +634,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B5EDDC-5ADB-4A4C-9736-3AC62D35C32F}">
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="18.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="18.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.88671875" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.5546875" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="3.88671875" customWidth="1"/>
-    <col min="14" max="14" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.6640625" customWidth="1"/>
-    <col min="17" max="17" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.6640625" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.5703125" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="3.85546875" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.7109375" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>18</v>
       </c>
@@ -678,7 +678,7 @@
       </c>
       <c r="Q1" s="10"/>
     </row>
-    <row r="2" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>24</v>
       </c>
@@ -716,7 +716,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -754,7 +754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -792,7 +792,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -830,7 +830,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -868,7 +868,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -906,7 +906,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -944,7 +944,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
@@ -976,7 +976,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G10" s="1" t="s">
         <v>13</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="J11" s="1" t="s">
         <v>13</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="J12" s="1" t="s">
         <v>14</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>17</v>
       </c>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="N14" s="10"/>
     </row>
-    <row r="15" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>24</v>
       </c>
@@ -1096,7 +1096,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>0</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -1342,7 +1342,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>2</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>34</v>
       </c>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="E28" s="8"/>
     </row>
-    <row r="29" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>5</v>
       </c>
@@ -1374,7 +1374,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>3</v>
       </c>
@@ -1388,7 +1388,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>13</v>
       </c>
@@ -1396,13 +1396,13 @@
         <v>35</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>16</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 31/07/2026 17:05:34,39
</commit_message>
<xml_diff>
--- a/Teletrabajo/Teletrabajo.xlsx
+++ b/Teletrabajo/Teletrabajo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Teletrabajo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C433DC3F-73FB-4639-96A7-86B318010383}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3471194-D1CC-4E32-9D95-A59E5E4E66C3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="42">
   <si>
     <t>Josue</t>
   </si>
@@ -159,6 +159,12 @@
   </si>
   <si>
     <t xml:space="preserve">Lunes </t>
+  </si>
+  <si>
+    <t>Semana del 3 al 7 Agosto</t>
+  </si>
+  <si>
+    <t>Semana del 10 al 14 Agosto</t>
   </si>
 </sst>
 </file>
@@ -1374,6 +1380,14 @@
         <v>32</v>
       </c>
       <c r="H28" s="8"/>
+      <c r="J28" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="K28" s="8"/>
+      <c r="M28" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="N28" s="8"/>
     </row>
     <row r="29" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
@@ -1394,6 +1408,18 @@
       <c r="H29" s="2" t="s">
         <v>39</v>
       </c>
+      <c r="J29" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="30" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
@@ -1414,6 +1440,18 @@
       <c r="H30" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="J30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
@@ -1434,6 +1472,18 @@
       <c r="H31" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="J31" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
@@ -1464,7 +1514,7 @@
       <c r="H34" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="P1:Q1"/>
@@ -1479,6 +1529,8 @@
     <mergeCell ref="M14:N14"/>
     <mergeCell ref="D28:E28"/>
     <mergeCell ref="G28:H28"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="M28:N28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion de datos - mié 19/08/2026 14:24:19,75
</commit_message>
<xml_diff>
--- a/Teletrabajo/Teletrabajo.xlsx
+++ b/Teletrabajo/Teletrabajo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Teletrabajo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CA5E9F9-7FD3-4F8A-A65A-79297BD1DF1A}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="13_ncr:1_{2BCD256D-733D-43D1-8F4C-E4456AFB0417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA8E7C56-5491-4CC6-8BC2-BC4230F75EF9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD785F99-1408-4CF3-B821-6417BD60C94A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="44">
   <si>
     <t>Josue</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>Semana del 17 al 21 Agosto</t>
+  </si>
+  <si>
+    <t>Semana del 24 al 28 Agosto</t>
   </si>
 </sst>
 </file>
@@ -1522,7 +1525,7 @@
       </c>
       <c r="B36" s="9"/>
       <c r="D36" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E36" s="9"/>
     </row>
@@ -1574,11 +1577,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A28:B28"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="D14:E14"/>
@@ -1590,6 +1588,11 @@
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="M14:N14"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="D28:E28"/>
     <mergeCell ref="G28:H28"/>
   </mergeCells>

</xml_diff>